<commit_message>
Add recipe import and fix the example import files
- Import page: Recipes, one row per raw material (Dish, Raw material, Quantity, Unit, For guests, Wastage %); each dish in the sheet gets its recipe in full, units convert (g/kg, ml/l, dozen/pcs), raw materials not in the inventory are listed and added in one click, and Undo restores the earlier recipes
- Better section guesses for new raw materials, including common Gujarati vegetable names
- Example files: sample rows now start right under the headings (they began at row 501), drop-downs kept; new 08 Recipes.xlsx; guide gains a Recipes page

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import-examples/01 Menu items.xlsx
+++ b/docs/import-examples/01 Menu items.xlsx
@@ -621,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L505"/>
+  <dimension ref="A1:L300"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -673,11 +673,196 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="5:8" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3">
+        <v>45</v>
+      </c>
+      <c r="J3">
+        <v>120</v>
+      </c>
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <v>40</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5">
+        <v>55</v>
+      </c>
+      <c r="J5">
+        <v>140</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6">
+        <v>40</v>
+      </c>
+      <c r="J6">
+        <v>110</v>
+      </c>
+      <c r="K6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="7" spans="5:8" x14ac:dyDescent="0.25"/>
     <row r="8" spans="5:8" x14ac:dyDescent="0.25"/>
     <row r="9" spans="5:8" x14ac:dyDescent="0.25"/>
@@ -972,414 +1157,24 @@
     <row r="298" spans="5:8" x14ac:dyDescent="0.25"/>
     <row r="299" spans="5:8" x14ac:dyDescent="0.25"/>
     <row r="300" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="301" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="302" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="303" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="304" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="305" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="306" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="307" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="308" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="309" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="310" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="311" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="312" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="313" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="314" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="315" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="316" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="317" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="318" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="319" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="320" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="321" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="322" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="323" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="324" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="325" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="326" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="327" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="328" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="329" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="330" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="331" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="332" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="333" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="334" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="335" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="336" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="337" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="338" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="339" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="340" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="341" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="342" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="343" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="344" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="345" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="346" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="347" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="348" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="349" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="350" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="351" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="352" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="353" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="354" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="355" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="356" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="357" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="358" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="359" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="360" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="361" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="362" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="363" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="364" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="365" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="366" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="367" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="368" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="369" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="370" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="371" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="372" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="373" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="374" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="375" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="376" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="377" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="378" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="379" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="380" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="381" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="382" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="383" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="384" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="385" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="386" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="387" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="388" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="389" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="390" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="391" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="392" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="393" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="394" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="395" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="396" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="397" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="398" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="399" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="400" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="401" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="402" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="403" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="404" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="405" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="406" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="407" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="408" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="409" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="410" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="411" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="412" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="413" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="414" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="415" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="416" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="417" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="418" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="419" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="420" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="421" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="422" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="423" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="424" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="425" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="426" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="427" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="428" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="429" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="430" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="431" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="432" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="433" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="434" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="435" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="436" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="437" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="438" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="439" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="440" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="441" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="442" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="443" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="444" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="445" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="446" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="447" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="448" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="449" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="450" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="451" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="452" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="453" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="454" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="455" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="456" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="457" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="458" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="459" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="460" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="461" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="462" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="463" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="464" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="465" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="466" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="467" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="468" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="469" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="470" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="471" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="472" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="473" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="474" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="475" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="476" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="477" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="478" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="479" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="480" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="481" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="482" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="483" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="484" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="485" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="486" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="487" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="488" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="489" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="490" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="491" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="492" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="493" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="494" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="495" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="496" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="497" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="498" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="499" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="500" spans="5:8" x14ac:dyDescent="0.25"/>
-    <row r="501" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A501" t="s">
-        <v>12</v>
-      </c>
-      <c r="B501" t="s">
-        <v>13</v>
-      </c>
-      <c r="C501" t="s">
-        <v>14</v>
-      </c>
-      <c r="D501" t="s">
-        <v>15</v>
-      </c>
-      <c r="E501" t="s">
-        <v>16</v>
-      </c>
-      <c r="F501" t="s">
-        <v>17</v>
-      </c>
-      <c r="G501" t="s">
-        <v>18</v>
-      </c>
-      <c r="H501" t="s">
-        <v>19</v>
-      </c>
-      <c r="I501">
-        <v>8</v>
-      </c>
-      <c r="J501">
-        <v>25</v>
-      </c>
-      <c r="K501" t="s">
-        <v>20</v>
-      </c>
-      <c r="L501" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="502" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A502" t="s">
-        <v>21</v>
-      </c>
-      <c r="B502" t="s">
-        <v>22</v>
-      </c>
-      <c r="C502" t="s">
-        <v>23</v>
-      </c>
-      <c r="D502" t="s">
-        <v>15</v>
-      </c>
-      <c r="E502" t="s">
-        <v>16</v>
-      </c>
-      <c r="F502" t="s">
-        <v>24</v>
-      </c>
-      <c r="G502" t="s">
-        <v>19</v>
-      </c>
-      <c r="H502" t="s">
-        <v>19</v>
-      </c>
-      <c r="I502">
-        <v>45</v>
-      </c>
-      <c r="J502">
-        <v>120</v>
-      </c>
-      <c r="K502" t="s">
-        <v>25</v>
-      </c>
-      <c r="L502" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="503" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A503" t="s">
-        <v>26</v>
-      </c>
-      <c r="B503" t="s">
-        <v>27</v>
-      </c>
-      <c r="C503" t="s">
-        <v>23</v>
-      </c>
-      <c r="D503" t="s">
-        <v>28</v>
-      </c>
-      <c r="E503" t="s">
-        <v>16</v>
-      </c>
-      <c r="F503" t="s">
-        <v>17</v>
-      </c>
-      <c r="G503" t="s">
-        <v>19</v>
-      </c>
-      <c r="H503" t="s">
-        <v>19</v>
-      </c>
-      <c r="I503">
-        <v>12</v>
-      </c>
-      <c r="J503">
-        <v>40</v>
-      </c>
-      <c r="K503" t="s">
-        <v>29</v>
-      </c>
-      <c r="L503" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="504" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A504" t="s">
-        <v>30</v>
-      </c>
-      <c r="B504" t="s">
-        <v>31</v>
-      </c>
-      <c r="C504" t="s">
-        <v>32</v>
-      </c>
-      <c r="D504" t="s">
-        <v>33</v>
-      </c>
-      <c r="E504" t="s">
-        <v>16</v>
-      </c>
-      <c r="F504" t="s">
-        <v>24</v>
-      </c>
-      <c r="G504" t="s">
-        <v>19</v>
-      </c>
-      <c r="H504" t="s">
-        <v>19</v>
-      </c>
-      <c r="I504">
-        <v>55</v>
-      </c>
-      <c r="J504">
-        <v>140</v>
-      </c>
-      <c r="K504" t="s">
-        <v>34</v>
-      </c>
-      <c r="L504" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="505" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A505" t="s">
-        <v>35</v>
-      </c>
-      <c r="B505" t="s">
-        <v>36</v>
-      </c>
-      <c r="C505" t="s">
-        <v>32</v>
-      </c>
-      <c r="D505" t="s">
-        <v>37</v>
-      </c>
-      <c r="E505" t="s">
-        <v>16</v>
-      </c>
-      <c r="F505" t="s">
-        <v>17</v>
-      </c>
-      <c r="G505" t="s">
-        <v>19</v>
-      </c>
-      <c r="H505" t="s">
-        <v>19</v>
-      </c>
-      <c r="I505">
-        <v>40</v>
-      </c>
-      <c r="J505">
-        <v>110</v>
-      </c>
-      <c r="K505" t="s">
-        <v>38</v>
-      </c>
-      <c r="L505" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Diet" error="Choose one of: Veg, Jain, Non-veg" sqref="E10:E500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Diet" error="Choose one of: Veg, Jain, Non-veg" sqref="E10:E300">
       <formula1>"Veg,Jain,Non-veg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Diet" error="Choose one of: Veg, Jain, Non-veg" sqref="E2:E500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Diet" error="Choose one of: Veg, Jain, Non-veg" sqref="E2:E300">
       <formula1>"Veg,Jain,Non-veg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Unit" error="Choose one of: plate, kg, piece, glass" sqref="G10:G500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Unit" error="Choose one of: plate, kg, piece, glass" sqref="G10:G300">
       <formula1>"plate,kg,piece,glass"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Unit" error="Choose one of: plate, kg, piece, glass" sqref="G2:G500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Unit" error="Choose one of: plate, kg, piece, glass" sqref="G2:G300">
       <formula1>"plate,kg,piece,glass"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Priced" error="Choose one of: plate, counter, flat" sqref="H10:H500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Priced" error="Choose one of: plate, counter, flat" sqref="H10:H300">
       <formula1>"plate,counter,flat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Priced" error="Choose one of: plate, counter, flat" sqref="H2:H500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Priced" error="Choose one of: plate, counter, flat" sqref="H2:H300">
       <formula1>"plate,counter,flat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Price staff and cutlery per event, fix 7-service bookings and multi-sheet imports
- Each event carries its own staff, cutlery and other charges, priced from new
  staff rates (Settings) and cutlery rent per piece, editable per booking;
  extras step, quotation, WhatsApp text and invoice group them by date with a
  total per event (migration 0018)
- Blank service names no longer block a booking; late services move to the
  next morning; services without a menu are flagged before saving
- Imports read every sheet of a workbook, fill down blank dish names, list
  held-back dishes, and save recipes in batches
- Rename Food type to Food Service Name and Service name to Event Name;
  menu item price is optional

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import-examples/01 Menu items.xlsx
+++ b/docs/import-examples/01 Menu items.xlsx
@@ -85,7 +85,7 @@
     <comment ref="J1" authorId="0">
       <text>
         <r>
-          <t>Required. Selling price per plate (or per counter), in rupees. Numbers only.</t>
+          <t>Optional. Selling price per plate (or per counter), in rupees. Numbers only. Can be left blank and set later.</t>
         </r>
       </text>
     </comment>
@@ -663,7 +663,7 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">

</xml_diff>